<commit_message>
arreglo vergara cochera 21
</commit_message>
<xml_diff>
--- a/VERGARA/Mayo/vergara MAYO.xlsx
+++ b/VERGARA/Mayo/vergara MAYO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\Desktop\RC CONSORCIO 2025\VERGARA\Mayo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistema\Desktop\rc-consorcio2025\VERGARA\Mayo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8545EB19-B4BE-46AD-ADC0-728153309E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0AAED02-C6CA-4BA8-96CB-0786DCB374B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="850" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="850" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="289">
   <si>
     <t>LIQUIDACION DE EXPENSAS</t>
   </si>
@@ -891,6 +891,9 @@
   </si>
   <si>
     <t>Santiago Tarragosa</t>
+  </si>
+  <si>
+    <t>HABIA PAGADO LOS 5300, SU DEUDA DEBE ESTAR EN 0</t>
   </si>
 </sst>
 </file>
@@ -898,15 +901,15 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="9">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;\ #,##0.00;[Red]\-&quot;$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0.00;[Red]\-&quot;$&quot;\ #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="_ &quot;$&quot;\ * #,##0.00_ ;_ &quot;$&quot;\ * \-#,##0.00_ ;_ &quot;$&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="167" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="_-&quot;$&quot;\ * #,##0.0_-;\-&quot;$&quot;\ * #,##0.0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="_-&quot;$&quot;\ * #,##0.0_-;\-&quot;$&quot;\ * #,##0.0_-;_-&quot;$&quot;\ * &quot;-&quot;?_-;_-@_-"/>
-    <numFmt numFmtId="170" formatCode="0.0"/>
-    <numFmt numFmtId="171" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_ &quot;$&quot;\ * #,##0.00_ ;_ &quot;$&quot;\ * \-#,##0.00_ ;_ &quot;$&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-&quot;$&quot;\ * #,##0.0_-;\-&quot;$&quot;\ * #,##0.0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-&quot;$&quot;\ * #,##0.0_-;\-&quot;$&quot;\ * #,##0.0_-;_-&quot;$&quot;\ * &quot;-&quot;?_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="25" x14ac:knownFonts="1">
     <font>
@@ -1511,10 +1514,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="221">
+  <cellXfs count="224">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1522,7 +1525,7 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="2" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1535,8 +1538,8 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1545,31 +1548,31 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="6" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="6" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="6" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="8" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="8" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1580,8 +1583,8 @@
     </xf>
     <xf numFmtId="16" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1602,19 +1605,19 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="9" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="20" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="20" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="20" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1635,35 +1638,35 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="5" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="22" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="23" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="9" fillId="4" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="22" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="23" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="9" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="9" fillId="4" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="23" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="9" fillId="4" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="23" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="23" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="23" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="6" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1671,12 +1674,12 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="23" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="23" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="19" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1687,18 +1690,18 @@
     <xf numFmtId="0" fontId="12" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="20" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="20" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="5" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="6" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1714,27 +1717,27 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="9" fillId="8" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="9" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="9" fillId="8" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="12" fillId="8" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="12" fillId="8" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1744,7 +1747,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="44" fontId="23" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1752,51 +1755,48 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="20" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="20" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="14" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="20" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="14" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="14" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="14" fillId="4" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="14" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="14" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="14" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="14" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="14" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="14" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="14" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1825,16 +1825,37 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1842,6 +1863,24 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="24" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1852,42 +1891,9 @@
     <xf numFmtId="0" fontId="12" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="24" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="0" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="20" fillId="11" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="14" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -2255,20 +2261,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M109"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.5703125" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" customWidth="1"/>
+    <col min="1" max="1" width="37.5546875" customWidth="1"/>
+    <col min="2" max="2" width="24.6640625" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="21.33203125" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="18.28515625" customWidth="1"/>
+    <col min="12" max="12" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="15"/>
       <c r="B1" s="68" t="s">
         <v>180</v>
@@ -2277,7 +2283,7 @@
       <c r="D1" s="68"/>
       <c r="E1" s="69"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="16"/>
       <c r="B2" s="136" t="s">
         <v>31</v>
@@ -2286,7 +2292,7 @@
       <c r="D2" s="136"/>
       <c r="E2" s="70"/>
     </row>
-    <row r="3" spans="1:5" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="16"/>
       <c r="B3" s="137" t="s">
         <v>213</v>
@@ -2297,7 +2303,7 @@
       </c>
       <c r="E3" s="70"/>
     </row>
-    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="17" t="s">
         <v>0</v>
       </c>
@@ -2308,18 +2314,18 @@
       <c r="D4" s="18"/>
       <c r="E4" s="19"/>
     </row>
-    <row r="5" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="16" t="s">
         <v>214</v>
       </c>
-      <c r="B5" s="185" t="s">
+      <c r="B5" s="199" t="s">
         <v>249</v>
       </c>
-      <c r="C5" s="185"/>
-      <c r="D5" s="185"/>
-      <c r="E5" s="186"/>
-    </row>
-    <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="199"/>
+      <c r="D5" s="199"/>
+      <c r="E5" s="200"/>
+    </row>
+    <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="17" t="s">
         <v>190</v>
       </c>
@@ -2330,57 +2336,57 @@
       </c>
       <c r="E6" s="19"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="188" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B8" s="202" t="s">
         <v>248</v>
       </c>
-      <c r="C8" s="188"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="188"/>
-      <c r="C9" s="188"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="188"/>
-      <c r="C10" s="188"/>
-    </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="187" t="s">
+      <c r="C8" s="202"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="202"/>
+      <c r="C9" s="202"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B10" s="202"/>
+      <c r="C10" s="202"/>
+    </row>
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="201" t="s">
         <v>189</v>
       </c>
-      <c r="B13" s="187"/>
-      <c r="C13" s="187"/>
-      <c r="D13" s="187"/>
-      <c r="E13" s="187"/>
-    </row>
-    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="187"/>
-      <c r="B14" s="187"/>
-      <c r="C14" s="187"/>
-      <c r="D14" s="187"/>
-      <c r="E14" s="187"/>
-    </row>
-    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="187"/>
-      <c r="B15" s="187"/>
-      <c r="C15" s="187"/>
-      <c r="D15" s="187"/>
-      <c r="E15" s="187"/>
-    </row>
-    <row r="16" spans="1:5" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="187"/>
-      <c r="B16" s="187"/>
-      <c r="C16" s="187"/>
-      <c r="D16" s="187"/>
-      <c r="E16" s="187"/>
-    </row>
-    <row r="17" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="201"/>
+      <c r="C13" s="201"/>
+      <c r="D13" s="201"/>
+      <c r="E13" s="201"/>
+    </row>
+    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="201"/>
+      <c r="B14" s="201"/>
+      <c r="C14" s="201"/>
+      <c r="D14" s="201"/>
+      <c r="E14" s="201"/>
+    </row>
+    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="201"/>
+      <c r="B15" s="201"/>
+      <c r="C15" s="201"/>
+      <c r="D15" s="201"/>
+      <c r="E15" s="201"/>
+    </row>
+    <row r="16" spans="1:5" ht="53.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="201"/>
+      <c r="B16" s="201"/>
+      <c r="C16" s="201"/>
+      <c r="D16" s="201"/>
+      <c r="E16" s="201"/>
+    </row>
+    <row r="17" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
     </row>
-    <row r="19" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>11</v>
       </c>
@@ -2389,7 +2395,7 @@
       <c r="D20" s="9"/>
       <c r="E20" s="14"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="33" t="s">
         <v>37</v>
       </c>
@@ -2398,42 +2404,42 @@
       <c r="D21" s="31"/>
       <c r="E21" s="31"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>188</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
-      <c r="D22" s="217">
+      <c r="D22" s="184">
         <v>598522.19999999995</v>
       </c>
       <c r="E22" s="90"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>186</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
-      <c r="D23" s="217">
+      <c r="D23" s="184">
         <v>-139605.89000000001</v>
       </c>
       <c r="E23" s="90"/>
       <c r="G23" s="20"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>187</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
-      <c r="D24" s="217">
+      <c r="D24" s="184">
         <v>0.69</v>
       </c>
       <c r="E24" s="90"/>
       <c r="G24" s="20"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="56" t="s">
         <v>38</v>
       </c>
@@ -2446,7 +2452,7 @@
       <c r="E25" s="91"/>
       <c r="G25" s="20"/>
     </row>
-    <row r="26" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="26" t="s">
         <v>1</v>
       </c>
@@ -2459,7 +2465,7 @@
       </c>
       <c r="F26" s="20"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="33" t="s">
         <v>23</v>
       </c>
@@ -2468,33 +2474,33 @@
       <c r="D27" s="34"/>
       <c r="E27" s="93"/>
     </row>
-    <row r="28" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="183" t="s">
+    <row r="28" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="188" t="s">
         <v>250</v>
       </c>
-      <c r="B28" s="184"/>
+      <c r="B28" s="189"/>
       <c r="C28" s="5"/>
-      <c r="D28" s="217">
+      <c r="D28" s="184">
         <v>31000</v>
       </c>
       <c r="E28" s="94" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="183" t="s">
+    <row r="29" spans="1:7" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="188" t="s">
         <v>252</v>
       </c>
-      <c r="B29" s="184"/>
+      <c r="B29" s="189"/>
       <c r="C29" s="5"/>
-      <c r="D29" s="217">
+      <c r="D29" s="184">
         <v>470000</v>
       </c>
       <c r="E29" s="94" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="26" t="s">
         <v>17</v>
       </c>
@@ -2506,7 +2512,7 @@
         <v>501000</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="31" t="s">
         <v>34</v>
       </c>
@@ -2515,30 +2521,30 @@
       <c r="D31" s="35"/>
       <c r="E31" s="67"/>
     </row>
-    <row r="32" spans="1:7" s="40" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" s="40" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="160" t="s">
         <v>277</v>
       </c>
       <c r="B32" s="154"/>
       <c r="C32" s="54"/>
-      <c r="D32" s="218">
+      <c r="D32" s="185">
         <v>70868</v>
       </c>
       <c r="E32" s="118"/>
       <c r="G32" s="159"/>
     </row>
-    <row r="33" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="183" t="s">
+    <row r="33" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="188" t="s">
         <v>278</v>
       </c>
-      <c r="B33" s="184"/>
+      <c r="B33" s="189"/>
       <c r="C33" s="54"/>
-      <c r="D33" s="219">
+      <c r="D33" s="186">
         <v>719.9</v>
       </c>
       <c r="E33" s="118"/>
     </row>
-    <row r="34" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="26" t="s">
         <v>2</v>
       </c>
@@ -2550,7 +2556,7 @@
         <v>71587.899999999994</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="33" t="s">
         <v>18</v>
       </c>
@@ -2559,13 +2565,13 @@
       <c r="D35" s="38"/>
       <c r="E35" s="97"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>47</v>
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="53"/>
-      <c r="D36" s="220">
+      <c r="D36" s="187">
         <v>295029.98</v>
       </c>
       <c r="E36" s="120" t="s">
@@ -2573,7 +2579,7 @@
       </c>
       <c r="G36" s="125"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>251</v>
       </c>
@@ -2588,7 +2594,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="str">
         <f>A37</f>
         <v>Sindicatos mes de MAYO</v>
@@ -2605,7 +2611,7 @@
         <v>Debito 12/05</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="str">
         <f>A38</f>
         <v>Sindicatos mes de MAYO</v>
@@ -2622,7 +2628,7 @@
         <v>Debito 12/05</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="26" t="s">
         <v>3</v>
       </c>
@@ -2634,7 +2640,7 @@
         <v>374947.26999999996</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="33" t="s">
         <v>20</v>
       </c>
@@ -2643,7 +2649,7 @@
       <c r="D41" s="38"/>
       <c r="E41" s="97"/>
     </row>
-    <row r="42" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>185</v>
       </c>
@@ -2652,7 +2658,7 @@
       <c r="D42" s="117"/>
       <c r="E42" s="103"/>
     </row>
-    <row r="43" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>273</v>
       </c>
@@ -2665,11 +2671,11 @@
         <v>274</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="183" t="s">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" s="188" t="s">
         <v>222</v>
       </c>
-      <c r="B44" s="184"/>
+      <c r="B44" s="189"/>
       <c r="C44" s="5"/>
       <c r="D44" s="117">
         <v>81423.929999999993</v>
@@ -2678,7 +2684,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="26" t="s">
         <v>4</v>
       </c>
@@ -2690,7 +2696,7 @@
         <v>131423.93</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="33" t="s">
         <v>19</v>
       </c>
@@ -2699,11 +2705,11 @@
       <c r="D46" s="37"/>
       <c r="E46" s="99"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="191" t="s">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="192" t="s">
         <v>271</v>
       </c>
-      <c r="B47" s="192"/>
+      <c r="B47" s="193"/>
       <c r="C47" s="65"/>
       <c r="D47" s="117">
         <v>84500</v>
@@ -2712,11 +2718,11 @@
         <v>259</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="191" t="s">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" s="192" t="s">
         <v>272</v>
       </c>
-      <c r="B48" s="192"/>
+      <c r="B48" s="193"/>
       <c r="C48" s="65"/>
       <c r="D48" s="117">
         <v>262099.86</v>
@@ -2726,7 +2732,7 @@
       </c>
       <c r="G48" s="140"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="155" t="s">
         <v>270</v>
       </c>
@@ -2739,7 +2745,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="155" t="s">
         <v>275</v>
       </c>
@@ -2752,11 +2758,11 @@
         <v>276</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="183" t="s">
+    <row r="51" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="188" t="s">
         <v>257</v>
       </c>
-      <c r="B51" s="184"/>
+      <c r="B51" s="189"/>
       <c r="C51" s="55"/>
       <c r="D51" s="117">
         <v>165000</v>
@@ -2765,11 +2771,11 @@
         <v>254</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="183" t="s">
+    <row r="52" spans="1:10" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="188" t="s">
         <v>281</v>
       </c>
-      <c r="B52" s="184"/>
+      <c r="B52" s="189"/>
       <c r="C52" s="55"/>
       <c r="D52" s="117">
         <v>450000</v>
@@ -2778,11 +2784,11 @@
         <v>260</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="183" t="s">
+    <row r="53" spans="1:10" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="188" t="s">
         <v>256</v>
       </c>
-      <c r="B53" s="184"/>
+      <c r="B53" s="189"/>
       <c r="C53" s="55"/>
       <c r="D53" s="117">
         <v>230000</v>
@@ -2791,7 +2797,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="143" t="s">
         <v>255</v>
       </c>
@@ -2804,11 +2810,11 @@
         <v>254</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="183" t="s">
+    <row r="55" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="188" t="s">
         <v>282</v>
       </c>
-      <c r="B55" s="184"/>
+      <c r="B55" s="189"/>
       <c r="C55" s="55"/>
       <c r="D55" s="117">
         <v>135000</v>
@@ -2817,7 +2823,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="143" t="s">
         <v>253</v>
       </c>
@@ -2830,11 +2836,11 @@
         <v>254</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="193" t="s">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A57" s="194" t="s">
         <v>264</v>
       </c>
-      <c r="B57" s="194"/>
+      <c r="B57" s="195"/>
       <c r="C57" s="5"/>
       <c r="D57" s="117">
         <v>110000</v>
@@ -2843,11 +2849,11 @@
         <v>263</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="183" t="s">
+    <row r="58" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="188" t="s">
         <v>261</v>
       </c>
-      <c r="B58" s="184"/>
+      <c r="B58" s="189"/>
       <c r="C58" s="5"/>
       <c r="D58" s="101">
         <v>150000</v>
@@ -2855,10 +2861,10 @@
       <c r="E58" s="157" t="s">
         <v>262</v>
       </c>
-      <c r="I58" s="183"/>
-      <c r="J58" s="184"/>
-    </row>
-    <row r="59" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I58" s="188"/>
+      <c r="J58" s="189"/>
+    </row>
+    <row r="59" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="26" t="s">
         <v>10</v>
       </c>
@@ -2870,7 +2876,7 @@
         <v>2702899.86</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="33" t="s">
         <v>13</v>
       </c>
@@ -2879,7 +2885,7 @@
       <c r="D60" s="28"/>
       <c r="E60" s="99"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
         <v>216</v>
       </c>
@@ -2891,7 +2897,7 @@
       </c>
       <c r="E61" s="107"/>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>217</v>
       </c>
@@ -2902,7 +2908,7 @@
       </c>
       <c r="E62" s="104"/>
     </row>
-    <row r="63" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="52" t="s">
         <v>17</v>
       </c>
@@ -2914,14 +2920,14 @@
         <v>168465.71000000002</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="5"/>
       <c r="B64" s="5"/>
       <c r="C64" s="5"/>
       <c r="D64" s="90"/>
       <c r="E64" s="109"/>
     </row>
-    <row r="65" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="29" t="s">
         <v>240</v>
       </c>
@@ -2930,14 +2936,14 @@
       <c r="D65" s="110"/>
       <c r="E65" s="142"/>
     </row>
-    <row r="66" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1"/>
       <c r="D66" s="111"/>
       <c r="E66" s="112"/>
       <c r="F66" s="45"/>
       <c r="G66" s="149"/>
     </row>
-    <row r="67" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
         <v>14</v>
       </c>
@@ -2950,15 +2956,15 @@
       </c>
       <c r="F67" s="140"/>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D68" s="111"/>
       <c r="E68" s="111"/>
     </row>
-    <row r="69" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D69" s="111"/>
       <c r="E69" s="111"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" s="11" t="s">
         <v>45</v>
       </c>
@@ -2967,11 +2973,11 @@
       <c r="D70" s="114"/>
       <c r="E70" s="115"/>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="183" t="s">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71" s="188" t="s">
         <v>258</v>
       </c>
-      <c r="B71" s="184"/>
+      <c r="B71" s="189"/>
       <c r="C71" s="5"/>
       <c r="D71" s="101">
         <v>304993.06</v>
@@ -2980,14 +2986,14 @@
         <v>268</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="100"/>
       <c r="B72" s="102"/>
       <c r="C72" s="5"/>
       <c r="D72" s="101"/>
       <c r="E72" s="98"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="50"/>
       <c r="B73" s="49"/>
       <c r="C73" s="49"/>
@@ -2997,19 +3003,19 @@
         <v>304993.06</v>
       </c>
     </row>
-    <row r="74" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="75" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="76" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="195" t="s">
+    <row r="74" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="75" spans="1:7" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="76" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A76" s="196" t="s">
         <v>279</v>
       </c>
-      <c r="B76" s="196"/>
-      <c r="C76" s="196"/>
-      <c r="D76" s="197"/>
+      <c r="B76" s="197"/>
+      <c r="C76" s="197"/>
+      <c r="D76" s="198"/>
       <c r="E76" s="150"/>
     </row>
-    <row r="77" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="78" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="78" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
         <v>24</v>
       </c>
@@ -3021,8 +3027,8 @@
         <v>304993.06</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="80" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="80" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A80" s="87" t="s">
         <v>15</v>
       </c>
@@ -3031,7 +3037,7 @@
         <v>4409241.67</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A81" s="87" t="s">
         <v>16</v>
       </c>
@@ -3040,7 +3046,7 @@
         <v>4409241.67</v>
       </c>
     </row>
-    <row r="82" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A82" s="87" t="s">
         <v>25</v>
       </c>
@@ -3049,7 +3055,7 @@
         <v>304993.06</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A83" s="87" t="s">
         <v>41</v>
       </c>
@@ -3058,15 +3064,15 @@
         <v>304993.06</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="73.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" ht="73.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="46" t="s">
         <v>36</v>
       </c>
       <c r="B85" s="126"/>
       <c r="C85" s="21"/>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="30" t="s">
         <v>179</v>
       </c>
@@ -3075,7 +3081,7 @@
       </c>
       <c r="C86" s="23"/>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="22" t="s">
         <v>9</v>
       </c>
@@ -3085,7 +3091,7 @@
       </c>
       <c r="C87" s="21"/>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="22" t="s">
         <v>43</v>
       </c>
@@ -3095,8 +3101,8 @@
       </c>
       <c r="C88" s="21"/>
     </row>
-    <row r="89" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="216" t="s">
+    <row r="89" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="183" t="s">
         <v>286</v>
       </c>
       <c r="B89" s="48">
@@ -3105,7 +3111,7 @@
       </c>
       <c r="C89" s="21"/>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" s="22" t="s">
         <v>285</v>
       </c>
@@ -3114,7 +3120,7 @@
       </c>
       <c r="C90" s="21"/>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" s="121" t="s">
         <v>46</v>
       </c>
@@ -3123,7 +3129,7 @@
       </c>
       <c r="C91" s="21"/>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="41" t="s">
         <v>26</v>
       </c>
@@ -3133,7 +3139,7 @@
       </c>
       <c r="C92" s="21"/>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="41" t="s">
         <v>218</v>
       </c>
@@ -3143,7 +3149,7 @@
       </c>
       <c r="C93" s="21"/>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="41" t="s">
         <v>219</v>
       </c>
@@ -3153,7 +3159,7 @@
       </c>
       <c r="C94" s="21"/>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="25" t="s">
         <v>27</v>
       </c>
@@ -3163,7 +3169,7 @@
       </c>
       <c r="C95" s="21"/>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="130" t="s">
         <v>10</v>
       </c>
@@ -3174,52 +3180,52 @@
       <c r="C96" s="24"/>
       <c r="D96" s="45"/>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B97" s="43"/>
       <c r="C97" s="24"/>
       <c r="D97" s="45"/>
       <c r="E97" s="127"/>
       <c r="F97" s="128"/>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B98" s="43"/>
       <c r="C98" s="24"/>
       <c r="D98" s="45"/>
       <c r="E98" s="127"/>
       <c r="F98" s="128"/>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A99" s="190" t="s">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A99" s="191" t="s">
         <v>35</v>
       </c>
-      <c r="B99" s="190"/>
-      <c r="C99" s="190"/>
-    </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A100" s="190"/>
-      <c r="B100" s="190"/>
-      <c r="C100" s="190"/>
-    </row>
-    <row r="101" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B99" s="191"/>
+      <c r="C99" s="191"/>
+    </row>
+    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A100" s="191"/>
+      <c r="B100" s="191"/>
+      <c r="C100" s="191"/>
+    </row>
+    <row r="101" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="54"/>
       <c r="B101" s="145"/>
       <c r="C101" s="36">
         <v>11948.17</v>
       </c>
     </row>
-    <row r="102" spans="1:13" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:13" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="54"/>
       <c r="B102" s="36"/>
       <c r="C102" s="36"/>
     </row>
-    <row r="103" spans="1:13" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:13" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="134"/>
       <c r="B103" s="36"/>
       <c r="C103" s="36">
         <v>61209</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A104" s="46" t="s">
         <v>10</v>
       </c>
@@ -3229,39 +3235,46 @@
       </c>
       <c r="C104" s="47"/>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
       <c r="M105" s="8"/>
     </row>
-    <row r="106" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="189"/>
-      <c r="B106" s="189"/>
-      <c r="C106" s="189"/>
-      <c r="D106" s="189"/>
-      <c r="E106" s="189"/>
-    </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A107" s="189"/>
-      <c r="B107" s="189"/>
-      <c r="C107" s="189"/>
-      <c r="D107" s="189"/>
-      <c r="E107" s="189"/>
-    </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A108" s="189"/>
-      <c r="B108" s="189"/>
-      <c r="C108" s="189"/>
-      <c r="D108" s="189"/>
-      <c r="E108" s="189"/>
-    </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A109" s="189"/>
-      <c r="B109" s="189"/>
-      <c r="C109" s="189"/>
-      <c r="D109" s="189"/>
-      <c r="E109" s="189"/>
+    <row r="106" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="190"/>
+      <c r="B106" s="190"/>
+      <c r="C106" s="190"/>
+      <c r="D106" s="190"/>
+      <c r="E106" s="190"/>
+    </row>
+    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A107" s="190"/>
+      <c r="B107" s="190"/>
+      <c r="C107" s="190"/>
+      <c r="D107" s="190"/>
+      <c r="E107" s="190"/>
+    </row>
+    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A108" s="190"/>
+      <c r="B108" s="190"/>
+      <c r="C108" s="190"/>
+      <c r="D108" s="190"/>
+      <c r="E108" s="190"/>
+    </row>
+    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A109" s="190"/>
+      <c r="B109" s="190"/>
+      <c r="C109" s="190"/>
+      <c r="D109" s="190"/>
+      <c r="E109" s="190"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="A13:E16"/>
+    <mergeCell ref="B8:C10"/>
     <mergeCell ref="I58:J58"/>
     <mergeCell ref="A106:E109"/>
     <mergeCell ref="A99:C100"/>
@@ -3275,13 +3288,6 @@
     <mergeCell ref="A48:B48"/>
     <mergeCell ref="A52:B52"/>
     <mergeCell ref="A55:B55"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="A13:E16"/>
-    <mergeCell ref="B8:C10"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3292,27 +3298,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:T100"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.28515625" hidden="1" customWidth="1"/>
-    <col min="2" max="3" width="4.28515625" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" customWidth="1"/>
-    <col min="5" max="5" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.42578125" customWidth="1"/>
-    <col min="7" max="7" width="14.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" customWidth="1"/>
-    <col min="9" max="9" width="10.5703125" customWidth="1"/>
-    <col min="10" max="11" width="9.5703125" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="15" width="11.7109375" customWidth="1"/>
-    <col min="16" max="16" width="14.7109375" customWidth="1"/>
-    <col min="17" max="17" width="14.28515625" customWidth="1"/>
-    <col min="18" max="18" width="10.42578125" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="4.33203125" hidden="1" customWidth="1"/>
+    <col min="2" max="3" width="4.33203125" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" customWidth="1"/>
+    <col min="5" max="5" width="32.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.44140625" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" customWidth="1"/>
+    <col min="9" max="9" width="10.5546875" customWidth="1"/>
+    <col min="10" max="11" width="9.5546875" customWidth="1"/>
+    <col min="12" max="12" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="11.6640625" customWidth="1"/>
+    <col min="16" max="16" width="14.6640625" customWidth="1"/>
+    <col min="17" max="17" width="14.33203125" customWidth="1"/>
+    <col min="18" max="18" width="10.44140625" hidden="1" customWidth="1"/>
     <col min="19" max="19" width="12" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -3320,10 +3326,10 @@
       <c r="E1" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="F1" s="207">
+      <c r="F1" s="203">
         <v>2102777.02</v>
       </c>
-      <c r="G1" s="207"/>
+      <c r="G1" s="203"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
       <c r="J1" s="6"/>
@@ -3331,19 +3337,19 @@
         <v>5</v>
       </c>
       <c r="L1" s="6"/>
-      <c r="M1" s="209">
+      <c r="M1" s="205">
         <f>P1</f>
         <v>3600000</v>
       </c>
-      <c r="N1" s="209"/>
+      <c r="N1" s="205"/>
       <c r="O1" s="144"/>
-      <c r="P1" s="214">
+      <c r="P1" s="213">
         <v>3600000</v>
       </c>
-      <c r="Q1" s="214"/>
+      <c r="Q1" s="213"/>
       <c r="R1" s="20"/>
     </row>
-    <row r="2" spans="1:20" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" ht="12.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -3351,105 +3357,105 @@
       <c r="E2" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="F2" s="208">
+      <c r="F2" s="204">
         <v>568429.56999999995</v>
       </c>
-      <c r="G2" s="208"/>
+      <c r="G2" s="204"/>
       <c r="H2" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="I2" s="213">
+      <c r="I2" s="212">
         <v>1200000</v>
       </c>
-      <c r="J2" s="213"/>
+      <c r="J2" s="212"/>
       <c r="K2" s="6" t="s">
         <v>241</v>
       </c>
       <c r="L2" s="6"/>
-      <c r="M2" s="213">
+      <c r="M2" s="212">
         <v>304993.06</v>
       </c>
-      <c r="N2" s="213"/>
+      <c r="N2" s="212"/>
       <c r="O2" s="146"/>
-      <c r="P2" s="215"/>
-      <c r="Q2" s="215"/>
-    </row>
-    <row r="3" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="198" t="s">
+      <c r="P2" s="214"/>
+      <c r="Q2" s="214"/>
+    </row>
+    <row r="3" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="215" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="122"/>
-      <c r="C3" s="200" t="s">
+      <c r="C3" s="208" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="200" t="s">
+      <c r="D3" s="208" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="200" t="s">
+      <c r="E3" s="208" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="200" t="s">
+      <c r="F3" s="208" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="202" t="s">
+      <c r="G3" s="210" t="s">
         <v>178</v>
       </c>
-      <c r="H3" s="200" t="s">
+      <c r="H3" s="208" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="204" t="s">
+      <c r="I3" s="218" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="202" t="s">
+      <c r="J3" s="210" t="s">
         <v>44</v>
       </c>
-      <c r="K3" s="202" t="str">
+      <c r="K3" s="210" t="str">
         <f>K2</f>
         <v>Plan de pago metrogas:</v>
       </c>
-      <c r="L3" s="202" t="s">
+      <c r="L3" s="210" t="s">
         <v>28</v>
       </c>
-      <c r="M3" s="202" t="s">
+      <c r="M3" s="210" t="s">
         <v>181</v>
       </c>
-      <c r="N3" s="202" t="s">
+      <c r="N3" s="210" t="s">
         <v>182</v>
       </c>
-      <c r="O3" s="202" t="s">
+      <c r="O3" s="210" t="s">
         <v>242</v>
       </c>
       <c r="P3" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="Q3" s="210" t="s">
+      <c r="Q3" s="206" t="s">
         <v>39</v>
       </c>
       <c r="T3" s="45"/>
     </row>
-    <row r="4" spans="1:20" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="199"/>
+    <row r="4" spans="1:20" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="216"/>
       <c r="B4" s="123"/>
-      <c r="C4" s="201"/>
-      <c r="D4" s="201"/>
-      <c r="E4" s="212"/>
-      <c r="F4" s="201"/>
-      <c r="G4" s="203"/>
-      <c r="H4" s="201"/>
-      <c r="I4" s="205"/>
-      <c r="J4" s="203"/>
-      <c r="K4" s="206"/>
-      <c r="L4" s="203"/>
-      <c r="M4" s="203"/>
-      <c r="N4" s="203"/>
-      <c r="O4" s="203"/>
+      <c r="C4" s="217"/>
+      <c r="D4" s="217"/>
+      <c r="E4" s="209"/>
+      <c r="F4" s="217"/>
+      <c r="G4" s="211"/>
+      <c r="H4" s="217"/>
+      <c r="I4" s="219"/>
+      <c r="J4" s="211"/>
+      <c r="K4" s="220"/>
+      <c r="L4" s="211"/>
+      <c r="M4" s="211"/>
+      <c r="N4" s="211"/>
+      <c r="O4" s="211"/>
       <c r="P4" s="59" t="str">
         <f>RESUMEN!B8</f>
         <v>VTO 16/06</v>
       </c>
-      <c r="Q4" s="211"/>
-    </row>
-    <row r="5" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q4" s="207"/>
+    </row>
+    <row r="5" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="62"/>
       <c r="B5" s="62" t="s">
         <v>48</v>
@@ -3512,7 +3518,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="62"/>
       <c r="B6" s="62" t="s">
         <v>50</v>
@@ -3576,7 +3582,7 @@
       </c>
       <c r="S6" s="45"/>
     </row>
-    <row r="7" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="62">
         <v>1</v>
       </c>
@@ -3640,7 +3646,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="62">
         <v>2</v>
       </c>
@@ -3703,7 +3709,7 @@
       </c>
       <c r="T8" s="45"/>
     </row>
-    <row r="9" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="62">
         <v>3</v>
       </c>
@@ -3771,7 +3777,7 @@
       </c>
       <c r="T9" s="45"/>
     </row>
-    <row r="10" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="62">
         <v>4</v>
       </c>
@@ -3838,7 +3844,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="62">
         <v>5</v>
       </c>
@@ -3903,7 +3909,7 @@
         <v>0.39</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="62">
         <v>6</v>
       </c>
@@ -3968,7 +3974,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="62">
         <v>7</v>
       </c>
@@ -4035,7 +4041,7 @@
         <v>0.41</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="62">
         <v>8</v>
       </c>
@@ -4102,7 +4108,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="62">
         <v>1</v>
       </c>
@@ -4169,7 +4175,7 @@
         <v>0.43</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="62">
         <v>1</v>
       </c>
@@ -4236,7 +4242,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="62">
         <v>2</v>
       </c>
@@ -4303,7 +4309,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="62">
         <v>2</v>
       </c>
@@ -4370,7 +4376,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="62">
         <v>3</v>
       </c>
@@ -4439,7 +4445,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="62">
         <v>3</v>
       </c>
@@ -4510,7 +4516,7 @@
       </c>
       <c r="T20" s="44"/>
     </row>
-    <row r="21" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="62">
         <v>4</v>
       </c>
@@ -4577,7 +4583,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="62">
         <v>4</v>
       </c>
@@ -4639,7 +4645,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="62">
         <v>5</v>
       </c>
@@ -4703,7 +4709,7 @@
         <v>0.51</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="62">
         <v>5</v>
       </c>
@@ -4770,7 +4776,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="62">
         <v>6</v>
       </c>
@@ -4834,7 +4840,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="26" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="62">
         <v>6</v>
       </c>
@@ -4901,7 +4907,7 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="62">
         <v>7</v>
       </c>
@@ -4968,7 +4974,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="28" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="62">
         <v>7</v>
       </c>
@@ -5035,7 +5041,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="62">
         <v>8</v>
       </c>
@@ -5100,7 +5106,7 @@
         <v>0.56999999999999995</v>
       </c>
     </row>
-    <row r="30" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="62">
         <v>8</v>
       </c>
@@ -5167,7 +5173,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="31" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="62">
         <v>9</v>
       </c>
@@ -5232,7 +5238,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="62">
         <v>9</v>
       </c>
@@ -5298,7 +5304,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="62">
         <v>10</v>
       </c>
@@ -5363,7 +5369,7 @@
         <v>0.61</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="62">
         <v>10</v>
       </c>
@@ -5430,7 +5436,7 @@
         <v>0.62</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" s="62">
         <v>11</v>
       </c>
@@ -5497,7 +5503,7 @@
         <v>0.63</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="62">
         <v>11</v>
       </c>
@@ -5564,7 +5570,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="62">
         <v>12</v>
       </c>
@@ -5631,7 +5637,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="38" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="62">
         <v>12</v>
       </c>
@@ -5695,7 +5701,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="39" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="62">
         <v>1</v>
       </c>
@@ -5762,7 +5768,7 @@
         <v>0.67</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="62">
         <v>1</v>
       </c>
@@ -5830,7 +5836,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="41" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="61">
         <v>1</v>
       </c>
@@ -5896,7 +5902,7 @@
         <v>0.69</v>
       </c>
     </row>
-    <row r="42" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="62">
         <v>2</v>
       </c>
@@ -5963,7 +5969,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="43" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="62">
         <v>2</v>
       </c>
@@ -6027,7 +6033,7 @@
         <v>0.71</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="62">
         <v>2</v>
       </c>
@@ -6091,7 +6097,7 @@
         <v>0.72</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="62">
         <v>3</v>
       </c>
@@ -6155,7 +6161,7 @@
         <v>0.73</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="62">
         <v>3</v>
       </c>
@@ -6222,7 +6228,7 @@
         <v>0.74</v>
       </c>
     </row>
-    <row r="47" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="62">
         <v>3</v>
       </c>
@@ -6290,7 +6296,7 @@
       </c>
       <c r="T47" s="152"/>
     </row>
-    <row r="48" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="62">
         <v>4</v>
       </c>
@@ -6357,7 +6363,7 @@
         <v>0.76</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="62">
         <v>4</v>
       </c>
@@ -6424,7 +6430,7 @@
         <v>0.77</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="62">
         <v>4</v>
       </c>
@@ -6488,7 +6494,7 @@
         <v>0.78</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="62">
         <v>5</v>
       </c>
@@ -6553,7 +6559,7 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="62">
         <v>5</v>
       </c>
@@ -6620,7 +6626,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="62">
         <v>5</v>
       </c>
@@ -6687,7 +6693,7 @@
         <v>0.81</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="62">
         <v>6</v>
       </c>
@@ -6752,7 +6758,7 @@
         <v>0.82</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="62">
         <v>6</v>
       </c>
@@ -6816,7 +6822,7 @@
         <v>0.83</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="62">
         <v>6</v>
       </c>
@@ -6881,7 +6887,7 @@
         <v>0.84</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="62">
         <v>7</v>
       </c>
@@ -6917,7 +6923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="62">
         <v>7</v>
       </c>
@@ -6953,7 +6959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="62">
         <v>7</v>
       </c>
@@ -7020,7 +7026,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="62">
         <v>8</v>
       </c>
@@ -7082,7 +7088,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="62">
         <v>8</v>
       </c>
@@ -7144,7 +7150,7 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="62">
         <v>8</v>
       </c>
@@ -7206,7 +7212,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="63" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="62">
         <v>9</v>
       </c>
@@ -7273,7 +7279,7 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="64" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="62">
         <v>9</v>
       </c>
@@ -7335,7 +7341,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="65" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="62">
         <v>9</v>
       </c>
@@ -7402,7 +7408,7 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="66" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="62">
         <v>10</v>
       </c>
@@ -7467,7 +7473,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="62">
         <v>10</v>
       </c>
@@ -7533,7 +7539,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="62">
         <v>10</v>
       </c>
@@ -7597,7 +7603,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="62">
         <v>11</v>
       </c>
@@ -7659,7 +7665,7 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="62">
         <v>11</v>
       </c>
@@ -7721,7 +7727,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="62">
         <v>11</v>
       </c>
@@ -7787,7 +7793,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="72" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="62"/>
       <c r="B72" s="81" t="s">
         <v>156</v>
@@ -7852,7 +7858,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="62"/>
       <c r="B73" s="81" t="s">
         <v>157</v>
@@ -7912,7 +7918,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="62"/>
       <c r="B74" s="81" t="s">
         <v>158</v>
@@ -7972,7 +7978,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="62"/>
       <c r="B75" s="81" t="s">
         <v>160</v>
@@ -8032,7 +8038,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="62"/>
       <c r="B76" s="81" t="s">
         <v>161</v>
@@ -8095,7 +8101,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="77" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="62"/>
       <c r="B77" s="81" t="s">
         <v>162</v>
@@ -8158,7 +8164,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="62"/>
       <c r="B78" s="81" t="s">
         <v>164</v>
@@ -8221,7 +8227,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="79" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="62"/>
       <c r="B79" s="81" t="s">
         <v>165</v>
@@ -8283,7 +8289,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="62"/>
       <c r="B80" s="81" t="s">
         <v>166</v>
@@ -8303,11 +8309,11 @@
       <c r="G80" s="72">
         <v>105752.06</v>
       </c>
-      <c r="H80" s="124">
+      <c r="H80" s="221">
         <f>100452.06</f>
         <v>100452.06</v>
       </c>
-      <c r="I80" s="73">
+      <c r="I80" s="222">
         <f t="shared" si="13"/>
         <v>5300</v>
       </c>
@@ -8347,8 +8353,11 @@
         <f t="shared" si="22"/>
         <v>0.06</v>
       </c>
-    </row>
-    <row r="81" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S80" s="223" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="81" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="62">
         <v>12</v>
       </c>
@@ -8410,7 +8419,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="62">
         <v>12</v>
       </c>
@@ -8472,7 +8481,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="83" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="62">
         <v>12</v>
       </c>
@@ -8537,7 +8546,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A84" s="62"/>
       <c r="B84" s="80" t="s">
         <v>171</v>
@@ -8597,7 +8606,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A85" s="62"/>
       <c r="B85" s="80" t="s">
         <v>172</v>
@@ -8662,7 +8671,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A86" s="62"/>
       <c r="B86" s="80" t="s">
         <v>173</v>
@@ -8727,7 +8736,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A87" s="62"/>
       <c r="B87" s="62" t="s">
         <v>174</v>
@@ -8790,7 +8799,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="88" spans="1:18" ht="22.5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A88" s="62"/>
       <c r="B88" s="62" t="s">
         <v>175</v>
@@ -8852,7 +8861,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A89" s="62"/>
       <c r="B89" s="62" t="s">
         <v>176</v>
@@ -8918,7 +8927,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A90" s="61"/>
       <c r="B90" s="61" t="s">
         <v>177</v>
@@ -8980,7 +8989,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="91" spans="1:18" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:18" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A91" s="62"/>
       <c r="B91" s="147"/>
       <c r="C91" s="147"/>
@@ -9000,7 +9009,7 @@
       <c r="Q91" s="170"/>
       <c r="R91" s="45"/>
     </row>
-    <row r="92" spans="1:18" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:18" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A92" s="85"/>
       <c r="B92" s="171"/>
       <c r="C92" s="172"/>
@@ -9055,105 +9064,116 @@
         <v>13568044.699999999</v>
       </c>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:18" x14ac:dyDescent="0.3">
       <c r="D93" s="51"/>
       <c r="E93" s="51"/>
     </row>
-    <row r="95" spans="1:18" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D95" s="189" t="str">
+    <row r="95" spans="1:18" ht="9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D95" s="190" t="str">
         <f>RESUMEN!A13</f>
         <v>ESTIMADOS PROPIETARIOS E INQUILINOS: POR FAVOR LOS QUE ABONAN EN PRIMER VENCIMIENTO ABONEN EL MONTO DE PRIMER VENCIMIENTO, ASI AGILIZAN LA LIQUIDACION, LES PEDIMOS ENCARECIDAMENTE QUE RESPETEN LOS CENTAVOS CORRESPONDIENTES A LA UNIDAD FUNCIONAL. ES DE CARÁCTER OBLIGATORIO INFORMAR VIA MAIL LAS EXPENSAS.</v>
       </c>
-      <c r="E95" s="189"/>
-      <c r="F95" s="189"/>
-      <c r="G95" s="189"/>
-      <c r="H95" s="189"/>
-      <c r="I95" s="189"/>
-      <c r="J95" s="189"/>
-      <c r="K95" s="189"/>
-      <c r="L95" s="189"/>
-      <c r="M95" s="189"/>
-      <c r="N95" s="189"/>
-      <c r="O95" s="189"/>
-      <c r="P95" s="189"/>
-    </row>
-    <row r="96" spans="1:18" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D96" s="189"/>
-      <c r="E96" s="189"/>
-      <c r="F96" s="189"/>
-      <c r="G96" s="189"/>
-      <c r="H96" s="189"/>
-      <c r="I96" s="189"/>
-      <c r="J96" s="189"/>
-      <c r="K96" s="189"/>
-      <c r="L96" s="189"/>
-      <c r="M96" s="189"/>
-      <c r="N96" s="189"/>
-      <c r="O96" s="189"/>
-      <c r="P96" s="189"/>
-    </row>
-    <row r="97" spans="4:16" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D97" s="189"/>
-      <c r="E97" s="189"/>
-      <c r="F97" s="189"/>
-      <c r="G97" s="189"/>
-      <c r="H97" s="189"/>
-      <c r="I97" s="189"/>
-      <c r="J97" s="189"/>
-      <c r="K97" s="189"/>
-      <c r="L97" s="189"/>
-      <c r="M97" s="189"/>
-      <c r="N97" s="189"/>
-      <c r="O97" s="189"/>
-      <c r="P97" s="189"/>
-    </row>
-    <row r="98" spans="4:16" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D98" s="189"/>
-      <c r="E98" s="189"/>
-      <c r="F98" s="189"/>
-      <c r="G98" s="189"/>
-      <c r="H98" s="189"/>
-      <c r="I98" s="189"/>
-      <c r="J98" s="189"/>
-      <c r="K98" s="189"/>
-      <c r="L98" s="189"/>
-      <c r="M98" s="189"/>
-      <c r="N98" s="189"/>
-      <c r="O98" s="189"/>
-      <c r="P98" s="189"/>
-    </row>
-    <row r="99" spans="4:16" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D99" s="189"/>
-      <c r="E99" s="189"/>
-      <c r="F99" s="189"/>
-      <c r="G99" s="189"/>
-      <c r="H99" s="189"/>
-      <c r="I99" s="189"/>
-      <c r="J99" s="189"/>
-      <c r="K99" s="189"/>
-      <c r="L99" s="189"/>
-      <c r="M99" s="189"/>
-      <c r="N99" s="189"/>
-      <c r="O99" s="189"/>
-      <c r="P99" s="189"/>
-    </row>
-    <row r="100" spans="4:16" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D100" s="189"/>
-      <c r="E100" s="189"/>
-      <c r="F100" s="189"/>
-      <c r="G100" s="189"/>
-      <c r="H100" s="189"/>
-      <c r="I100" s="189"/>
-      <c r="J100" s="189"/>
-      <c r="K100" s="189"/>
-      <c r="L100" s="189"/>
-      <c r="M100" s="189"/>
-      <c r="N100" s="189"/>
-      <c r="O100" s="189"/>
-      <c r="P100" s="189"/>
+      <c r="E95" s="190"/>
+      <c r="F95" s="190"/>
+      <c r="G95" s="190"/>
+      <c r="H95" s="190"/>
+      <c r="I95" s="190"/>
+      <c r="J95" s="190"/>
+      <c r="K95" s="190"/>
+      <c r="L95" s="190"/>
+      <c r="M95" s="190"/>
+      <c r="N95" s="190"/>
+      <c r="O95" s="190"/>
+      <c r="P95" s="190"/>
+    </row>
+    <row r="96" spans="1:18" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D96" s="190"/>
+      <c r="E96" s="190"/>
+      <c r="F96" s="190"/>
+      <c r="G96" s="190"/>
+      <c r="H96" s="190"/>
+      <c r="I96" s="190"/>
+      <c r="J96" s="190"/>
+      <c r="K96" s="190"/>
+      <c r="L96" s="190"/>
+      <c r="M96" s="190"/>
+      <c r="N96" s="190"/>
+      <c r="O96" s="190"/>
+      <c r="P96" s="190"/>
+    </row>
+    <row r="97" spans="4:16" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D97" s="190"/>
+      <c r="E97" s="190"/>
+      <c r="F97" s="190"/>
+      <c r="G97" s="190"/>
+      <c r="H97" s="190"/>
+      <c r="I97" s="190"/>
+      <c r="J97" s="190"/>
+      <c r="K97" s="190"/>
+      <c r="L97" s="190"/>
+      <c r="M97" s="190"/>
+      <c r="N97" s="190"/>
+      <c r="O97" s="190"/>
+      <c r="P97" s="190"/>
+    </row>
+    <row r="98" spans="4:16" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D98" s="190"/>
+      <c r="E98" s="190"/>
+      <c r="F98" s="190"/>
+      <c r="G98" s="190"/>
+      <c r="H98" s="190"/>
+      <c r="I98" s="190"/>
+      <c r="J98" s="190"/>
+      <c r="K98" s="190"/>
+      <c r="L98" s="190"/>
+      <c r="M98" s="190"/>
+      <c r="N98" s="190"/>
+      <c r="O98" s="190"/>
+      <c r="P98" s="190"/>
+    </row>
+    <row r="99" spans="4:16" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D99" s="190"/>
+      <c r="E99" s="190"/>
+      <c r="F99" s="190"/>
+      <c r="G99" s="190"/>
+      <c r="H99" s="190"/>
+      <c r="I99" s="190"/>
+      <c r="J99" s="190"/>
+      <c r="K99" s="190"/>
+      <c r="L99" s="190"/>
+      <c r="M99" s="190"/>
+      <c r="N99" s="190"/>
+      <c r="O99" s="190"/>
+      <c r="P99" s="190"/>
+    </row>
+    <row r="100" spans="4:16" ht="60.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D100" s="190"/>
+      <c r="E100" s="190"/>
+      <c r="F100" s="190"/>
+      <c r="G100" s="190"/>
+      <c r="H100" s="190"/>
+      <c r="I100" s="190"/>
+      <c r="J100" s="190"/>
+      <c r="K100" s="190"/>
+      <c r="L100" s="190"/>
+      <c r="M100" s="190"/>
+      <c r="N100" s="190"/>
+      <c r="O100" s="190"/>
+      <c r="P100" s="190"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="L3:L4"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="M1:N1"/>
@@ -9166,17 +9186,6 @@
     <mergeCell ref="P1:Q1"/>
     <mergeCell ref="P2:Q2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="L3:L4"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="3" orientation="landscape" r:id="rId1"/>

</xml_diff>